<commit_message>
vault backup: 2026-10-15 14:04:30
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
+++ b/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.obsidian\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C9F6019-2FAC-4A2F-BF9A-F1EE58A8E54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF202E2E-3E40-41C6-A83F-ABDC910BBF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24900" yWindow="-1110" windowWidth="23790" windowHeight="14970" tabRatio="837" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" tabRatio="221" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="국디마" sheetId="15" r:id="rId1"/>
+    <sheet name="국디마 업데이트" sheetId="17" r:id="rId1"/>
+    <sheet name="국디마" sheetId="15" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">국디마!$B$3:$J$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">국디마!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">국디마!$B$3:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'국디마 업데이트'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">국디마!$A$1:$I$5</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="172">
   <si>
     <t>일련
 번호</t>
@@ -431,13 +433,287 @@
   </si>
   <si>
     <t>서초구 고터·세빛 관광특구</t>
+  </si>
+  <si>
+    <t>도메인</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://goodsti.com/</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kr.canon/main</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>추가 정보</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.utour.go.kr/intro.web</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://chilgok.kccf.or.kr:444/</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>주소</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 영등포구 국회대로68길 23, 6층(정원빌딩)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울특별시 강남구 테헤란로 607 (삼성동) </t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경상남도 통영시 통영해안로 515(무전동)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.pocheon.go.kr/ktour/index.do</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경기도 포천시 중앙로 87(신읍동)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.cbtour.or.kr/home/main.php</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>충청북도 청주시 상당구 상당로59번길 15 1층</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://dgfca.or.kr/main</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>대구광역시 달서구 공원순환로 201 대구문화예술진흥원</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.yeongju.go.kr/open_content/tour/index.do#</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경상북도 영주시 시청로 1, 영주시청 관광진흥과</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.yeodam.kr/product/product_view?id=TP20241213048</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://mom-mom.net/company</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://nonunbub.com/home</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>인천광역시 연수구 컨벤시아대로 204, 1층 108호</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.swtour.co.kr/</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://ktx7788.com/travel/index.html?itr=1</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.ktxtour.co.kr/index.asp</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.everland.com/everland/home/main</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kna.forest.go.kr/kfsweb/kfs/subIdx/Index.do?mn=UKNA</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경기도 포천시 소흘읍 광릉수목원로 509</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.koroad.or.kr/</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>강원특별자치도 원주시 혁신로 2 (반곡동)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>한국도로교통공단으로 추정</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.h-point.co.kr/cu/main/index.nhd</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>현대백화점그룹의 통합 라이프스타일 멤버십 플랫폼</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경상북도 칠곡군 왜관읍 2번도로길 23</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 중구 소공로 88(소공동) 한진빌딩 신관 9층</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 강남구 테헤란로52길 17 ES타워 8층</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 마포구 양화로 12길 24 (선진빌딩) 4층</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 종로구 삼봉로 95 대성스카이렉스 401호</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 용산구 한강대로 257, 7층(갈월동, 청룡빌딩)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 강남구 테헤란로98길 12</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.koagi.or.kr/www/intro.do</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>세종특별자치시 수목원로 136</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.seocho.go.kr/site/seocho/04/10405180900002025111103.jsp</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 서초구 남부순환로 2584 (서초동)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>서초구청 문화행정국 문화관광과 관광팀 주무관</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>사업본부 수목원사업실 담당주임 (국민평가단 운영)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>산림청 국립수목원 국립수목원 산림생물보전연구과 연구사</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>경기도 용인시 처인구 포곡읍 에버랜드로 199</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>해밀여행사 커뮤니티 담당, 콘텐츠 제작 등</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>노는법 호스트 활동  '로컬에서 1박2일 노는법' 프로그램을 운영</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>원더윅스컴퍼니의 전략총괄이사(CSO), 키즈 프렌들리 여행 및 
+숙박 상품 기획, 야놀자클라우드 등 주요 파트너와의 제휴 및
+'맘맘 체크인'·'맘맘 쇼케이스' 사업 운영</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>여행을 담다</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>관광마케팅팀 인센티브 담당자</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>대구문화예술진흥원 관광본부에서 운영하는 대구관광 공식 
+유튜브 채널('비짓대구') 및 관련 사업(예: SNS 채널 운영 제안서
+ 평가위원 모집 등)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>충북문화재단 마이스뷰로(충북 MICE 얼라이언스 운영 담당
+충북 MICE 얼라이언스는 2026년 기준 91개 기업·기관이 참여하는 
+협력 네트워크로 확대되었으며, 관련 실무 및 행사가 운영</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>트래킹 커뮤니티 담당으로 추정</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>대구석 여행기사 콘텐츠 관련, 포천시 지역문화정보 운영 관련</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">문화관광과 관광진흥팀 </t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>통영U투어 통영시청 관광지원과, 대구석 여행기사 콘텐츠 관련</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>그룹 분류</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>G5</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>지자체</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>G6</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>G7</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>책임연구원 FGI 조사진행</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP활용? 삼성물산 에버랜드 홍보팀 재직 등 (동화작가?)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>컨택현황</t>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,8 +794,92 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="DejaVu Sans"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,8 +898,38 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFD6D6D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -582,16 +972,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -655,10 +1078,156 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="7" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="8" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="8" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="하이퍼링크" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="38">
     <dxf>
@@ -1585,6 +2154,962 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C0977FD-8DA5-49F0-81F0-04370578922E}">
+  <sheetPr>
+    <tabColor rgb="FFB9CDE5"/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr defaultRowHeight="12"/>
+  <cols>
+    <col min="1" max="1" width="4.5" style="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.375" style="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.25" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.625" style="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.375" style="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.875" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.125" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.125" style="19" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.625" style="19" customWidth="1"/>
+    <col min="14" max="14" width="15.5" style="19" customWidth="1"/>
+    <col min="15" max="16384" width="9" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="30.75" customHeight="1">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="N1" s="18" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="13.5">
+      <c r="A2" s="24">
+        <v>9</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="L2" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N2" s="30"/>
+    </row>
+    <row r="3" spans="1:14" ht="40.5">
+      <c r="A3" s="24">
+        <v>10</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="H3" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="I3" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K3" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="L3" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N3" s="30"/>
+    </row>
+    <row r="4" spans="1:14" ht="13.5">
+      <c r="A4" s="24">
+        <v>11</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="I4" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L4" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N4" s="30"/>
+    </row>
+    <row r="5" spans="1:14" ht="13.5">
+      <c r="A5" s="24">
+        <v>12</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="J5" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="K5" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="M5" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N5" s="30"/>
+    </row>
+    <row r="6" spans="1:14" ht="13.5">
+      <c r="A6" s="24">
+        <v>13</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="L6" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N6" s="30"/>
+    </row>
+    <row r="7" spans="1:14" ht="13.5">
+      <c r="A7" s="24">
+        <v>14</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="H7" s="27"/>
+      <c r="I7" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="J7" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="N7" s="30"/>
+    </row>
+    <row r="8" spans="1:14" ht="13.5">
+      <c r="A8" s="33">
+        <v>3</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="H8" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="I8" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="M8" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N8" s="40"/>
+    </row>
+    <row r="9" spans="1:14" ht="13.5">
+      <c r="A9" s="33">
+        <v>4</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="G9" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="H9" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="M9" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N9" s="40"/>
+    </row>
+    <row r="10" spans="1:14" ht="13.5">
+      <c r="A10" s="42">
+        <v>5</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="G10" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="H10" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="I10" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="J10" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="L10" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="M10" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N10" s="40"/>
+    </row>
+    <row r="11" spans="1:14" ht="13.5">
+      <c r="A11" s="33">
+        <v>8</v>
+      </c>
+      <c r="B11" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="G11" s="48" t="s">
+        <v>122</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="I11" s="34" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="M11" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N11" s="40"/>
+    </row>
+    <row r="12" spans="1:14" ht="13.5">
+      <c r="A12" s="33">
+        <v>20</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="I12" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="K12" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="L12" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="M12" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="N12" s="49"/>
+    </row>
+    <row r="13" spans="1:14" ht="40.5">
+      <c r="A13" s="33">
+        <v>6</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="G13" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="H13" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="I13" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="L13" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="M13" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N13" s="40"/>
+    </row>
+    <row r="14" spans="1:14" ht="40.5">
+      <c r="A14" s="42">
+        <v>7</v>
+      </c>
+      <c r="B14" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="45" t="s">
+        <v>120</v>
+      </c>
+      <c r="H14" s="47" t="s">
+        <v>158</v>
+      </c>
+      <c r="I14" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="K14" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="L14" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="M14" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N14" s="40"/>
+    </row>
+    <row r="15" spans="1:14" ht="13.5">
+      <c r="A15" s="33">
+        <v>16</v>
+      </c>
+      <c r="B15" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="G15" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="H15" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="I15" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="K15" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="L15" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="M15" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N15" s="40"/>
+    </row>
+    <row r="16" spans="1:14" ht="13.5">
+      <c r="A16" s="33">
+        <v>17</v>
+      </c>
+      <c r="B16" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="I16" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="J16" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="K16" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="L16" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="M16" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="N16" s="40"/>
+    </row>
+    <row r="17" spans="1:14" ht="13.5">
+      <c r="A17" s="33">
+        <v>19</v>
+      </c>
+      <c r="B17" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="H17" s="37" t="s">
+        <v>150</v>
+      </c>
+      <c r="I17" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="J17" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K17" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="L17" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="M17" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="N17" s="49"/>
+    </row>
+    <row r="18" spans="1:14" ht="13.5">
+      <c r="A18" s="50">
+        <v>1</v>
+      </c>
+      <c r="B18" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" s="53" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="I18" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="J18" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" s="54" t="s">
+        <v>41</v>
+      </c>
+      <c r="L18" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="M18" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="N18" s="56"/>
+    </row>
+    <row r="19" spans="1:14" ht="13.5">
+      <c r="A19" s="50">
+        <v>2</v>
+      </c>
+      <c r="B19" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="52" t="s">
+        <v>107</v>
+      </c>
+      <c r="G19" s="53" t="s">
+        <v>113</v>
+      </c>
+      <c r="H19" s="52"/>
+      <c r="I19" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="J19" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="K19" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="L19" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="M19" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="N19" s="56"/>
+    </row>
+    <row r="20" spans="1:14" ht="13.5">
+      <c r="A20" s="50">
+        <v>15</v>
+      </c>
+      <c r="B20" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="51" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="G20" s="57" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="57" t="s">
+        <v>170</v>
+      </c>
+      <c r="I20" s="51" t="s">
+        <v>75</v>
+      </c>
+      <c r="J20" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="K20" s="54" t="s">
+        <v>87</v>
+      </c>
+      <c r="L20" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="M20" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="N20" s="56"/>
+    </row>
+    <row r="21" spans="1:14" ht="13.5">
+      <c r="A21" s="50">
+        <v>18</v>
+      </c>
+      <c r="B21" s="51" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="52" t="s">
+        <v>136</v>
+      </c>
+      <c r="G21" s="57" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" s="57" t="s">
+        <v>137</v>
+      </c>
+      <c r="I21" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="J21" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="K21" s="54" t="s">
+        <v>82</v>
+      </c>
+      <c r="L21" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="M21" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="N21" s="56"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N21" xr:uid="{2C0977FD-8DA5-49F0-81F0-04370578922E}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M23">
+    <sortCondition ref="M2:M23"/>
+    <sortCondition descending="1" ref="L2:L23"/>
+  </sortState>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="일련번호는 숫자로만 입력해주세요" prompt="일련번호는 숫자로만 입력해주세요" sqref="A2:A21" xr:uid="{5BDD78A4-C830-42D6-990C-52C389E62621}">
+      <formula1>0</formula1>
+      <formula2>99999999</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B21" xr:uid="{EA74545C-42B2-43CA-8A63-D4CABA33B41E}">
+      <formula1>"웹앱, SNS, 부스터, 오디"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D21" xr:uid="{768701E3-4ABE-49F3-97EC-B303DF2E5C8C}">
+      <formula1>"민간기업, 공공기관, 지자체"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="K13" r:id="rId1" xr:uid="{6859F9D7-C884-4203-B104-5C99CBD74201}"/>
+    <hyperlink ref="K14" r:id="rId2" xr:uid="{4CBFA95E-DAB7-4A62-9A9B-00CB9B43D14C}"/>
+    <hyperlink ref="K11" r:id="rId3" xr:uid="{11D31868-283D-4AF6-819E-A4CBB56B2492}"/>
+    <hyperlink ref="K19" r:id="rId4" xr:uid="{8FDF2054-CBCD-492F-9D65-99D3B3070ECB}"/>
+    <hyperlink ref="K21" r:id="rId5" xr:uid="{22645371-EC73-42A8-84CF-DCC4E3110820}"/>
+    <hyperlink ref="K15" r:id="rId6" xr:uid="{8ABF9306-138C-4479-BBD5-61F0C132B701}"/>
+    <hyperlink ref="K2" r:id="rId7" xr:uid="{023F2B73-17F2-46F8-A1AF-E178C5DFA648}"/>
+    <hyperlink ref="F18" r:id="rId8" xr:uid="{AEF8ED46-23B5-4C0A-A76B-3065CDEE582D}"/>
+    <hyperlink ref="F19" r:id="rId9" xr:uid="{94997D22-32E9-4AA2-A0B8-50A742B5872B}"/>
+    <hyperlink ref="F8" r:id="rId10" xr:uid="{AD0F59FA-B931-4120-9E68-2DDDB5A36638}"/>
+    <hyperlink ref="F9" r:id="rId11" xr:uid="{686514B7-7D08-4826-BD66-1F60689639BD}"/>
+    <hyperlink ref="F10" r:id="rId12" xr:uid="{83EC6681-68F6-4B1B-8D78-46E4F35C93BB}"/>
+    <hyperlink ref="F13" r:id="rId13" xr:uid="{9E34E430-20D7-4DFE-B44C-47C14853010B}"/>
+    <hyperlink ref="F14" r:id="rId14" xr:uid="{998E77A1-0DB4-4BD7-82C4-119D0F06CDAA}"/>
+    <hyperlink ref="F11" r:id="rId15" xr:uid="{E7000206-83A3-4C8A-8500-1FB173B6A0B1}"/>
+    <hyperlink ref="F2" r:id="rId16" xr:uid="{649535E5-E033-4C30-B99C-5F2AC4AA5FD3}"/>
+    <hyperlink ref="F3" r:id="rId17" xr:uid="{B5755B37-EE1A-4BA8-B768-30E5A36D5C16}"/>
+    <hyperlink ref="F4" r:id="rId18" xr:uid="{138E125E-3379-46F6-8895-F162234B718E}"/>
+    <hyperlink ref="F5" r:id="rId19" xr:uid="{D24708D2-70FC-40E6-8CCC-35F37EA13FE6}"/>
+    <hyperlink ref="F6" r:id="rId20" xr:uid="{4221549C-0A8E-415F-956C-E0737C7573AA}"/>
+    <hyperlink ref="F7" r:id="rId21" xr:uid="{461D595F-6F60-406F-93C8-F0093527C2CB}"/>
+    <hyperlink ref="F20" r:id="rId22" xr:uid="{F368191F-0112-4449-8A48-E5C169B0323A}"/>
+    <hyperlink ref="F15" r:id="rId23" xr:uid="{1088D30B-5B4E-40BF-BF57-D3B497CC6760}"/>
+    <hyperlink ref="F16" r:id="rId24" xr:uid="{9649CD7C-D06F-4FE5-8593-DF82F79F326C}"/>
+    <hyperlink ref="F21" r:id="rId25" xr:uid="{679D3E72-9279-47D3-91CD-99C8523C3DEA}"/>
+    <hyperlink ref="F17" r:id="rId26" xr:uid="{92BCAE65-3EDC-4C7F-8029-BAF238008192}"/>
+    <hyperlink ref="F12" r:id="rId27" xr:uid="{22EC201B-FDE9-42C4-9650-3D081C48AAC0}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFB9CDE5"/>

</xml_diff>

<commit_message>
docs: add 20261015 FGI industry recruiting progress note and sync vault structure
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
+++ b/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.obsidian\50_FGI\FGI 업계\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF202E2E-3E40-41C6-A83F-ABDC910BBF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3045BADB-B8AE-4BD1-A4BE-A0CE561D7D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" tabRatio="221" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,8 +21,19 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'국디마 업데이트'!$A$1:$N$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">국디마!$A$1:$I$5</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -31,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="181">
   <si>
     <t>일련
 번호</t>
@@ -705,7 +716,43 @@
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
-    <t>컨택현황</t>
+    <t>메일 발송 완료</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>한국수목원정원관리원</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>조형진</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>puruda@koagi.or.kr</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>메일 정보 대기</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>seo1@swtour.co.kr</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>1차 참가의향 메일발송</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>1차 메일 회신</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>불참 확정</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>1차 전화컨택</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -713,7 +760,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -857,13 +904,6 @@
       <charset val="129"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
@@ -878,8 +918,23 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -925,6 +980,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1014,7 +1075,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1081,7 +1142,7 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1112,10 +1173,7 @@
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1126,9 +1184,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
@@ -1149,19 +1204,13 @@
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
@@ -1209,10 +1258,7 @@
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1222,6 +1268,60 @@
     <xf numFmtId="49" fontId="13" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="2" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2158,12 +2258,12 @@
   <sheetPr>
     <tabColor rgb="FFB9CDE5"/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="4.5" style="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.375" style="19" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.25" style="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.25" style="19" customWidth="1"/>
     <col min="4" max="4" width="8" style="19" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.625" style="19" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="60.375" style="19" bestFit="1" customWidth="1"/>
@@ -2173,11 +2273,13 @@
     <col min="10" max="10" width="12.625" style="19" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23.125" style="19" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="10.625" style="19" customWidth="1"/>
-    <col min="14" max="14" width="15.5" style="19" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="19"/>
+    <col min="14" max="14" width="20.25" style="19" customWidth="1"/>
+    <col min="15" max="15" width="15" style="62" customWidth="1"/>
+    <col min="16" max="16" width="11.375" style="19" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30.75" customHeight="1">
+    <row r="1" spans="1:16" ht="30.75" customHeight="1">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -2218,10 +2320,16 @@
         <v>164</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="13.5">
+        <v>177</v>
+      </c>
+      <c r="O1" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="P1" s="66" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="16.5">
       <c r="A2" s="24">
         <v>9</v>
       </c>
@@ -2252,18 +2360,22 @@
       <c r="J2" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="L2" s="29" t="s">
+      <c r="L2" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="M2" s="30" t="s">
+      <c r="M2" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N2" s="30"/>
-    </row>
-    <row r="3" spans="1:14" ht="40.5">
+      <c r="N2" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="O2" s="63"/>
+      <c r="P2" s="67"/>
+    </row>
+    <row r="3" spans="1:16" ht="40.5">
       <c r="A3" s="24">
         <v>10</v>
       </c>
@@ -2285,7 +2397,7 @@
       <c r="G3" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="30" t="s">
         <v>155</v>
       </c>
       <c r="I3" s="25" t="s">
@@ -2294,18 +2406,22 @@
       <c r="J3" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="28" t="s">
+      <c r="K3" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="L3" s="29" t="s">
+      <c r="L3" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="M3" s="30" t="s">
+      <c r="M3" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N3" s="30"/>
-    </row>
-    <row r="4" spans="1:14" ht="13.5">
+      <c r="N3" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="O3" s="63"/>
+      <c r="P3" s="67"/>
+    </row>
+    <row r="4" spans="1:16" ht="16.5">
       <c r="A4" s="24">
         <v>11</v>
       </c>
@@ -2336,18 +2452,22 @@
       <c r="J4" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="L4" s="29" t="s">
+      <c r="L4" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="M4" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N4" s="30"/>
-    </row>
-    <row r="5" spans="1:14" ht="13.5">
+      <c r="N4" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="O4" s="63"/>
+      <c r="P4" s="67"/>
+    </row>
+    <row r="5" spans="1:16" ht="16.5">
       <c r="A5" s="24">
         <v>12</v>
       </c>
@@ -2378,18 +2498,22 @@
       <c r="J5" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="K5" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="L5" s="29" t="s">
+      <c r="K5" s="54" t="s">
+        <v>176</v>
+      </c>
+      <c r="L5" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="M5" s="30" t="s">
+      <c r="M5" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N5" s="30"/>
-    </row>
-    <row r="6" spans="1:14" ht="13.5">
+      <c r="N5" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="O5" s="63"/>
+      <c r="P5" s="67"/>
+    </row>
+    <row r="6" spans="1:16" ht="16.5">
       <c r="A6" s="24">
         <v>13</v>
       </c>
@@ -2420,18 +2544,22 @@
       <c r="J6" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="K6" s="28" t="s">
+      <c r="K6" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="L6" s="29" t="s">
+      <c r="L6" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="M6" s="30" t="s">
+      <c r="M6" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N6" s="30"/>
-    </row>
-    <row r="7" spans="1:14" ht="13.5">
+      <c r="N6" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="O6" s="63"/>
+      <c r="P6" s="67"/>
+    </row>
+    <row r="7" spans="1:16" ht="13.5">
       <c r="A7" s="24">
         <v>14</v>
       </c>
@@ -2463,602 +2591,665 @@
       <c r="K7" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="29" t="s">
+      <c r="L7" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="M7" s="30" t="s">
+      <c r="M7" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="N7" s="30"/>
-    </row>
-    <row r="8" spans="1:14" ht="13.5">
-      <c r="A8" s="33">
+      <c r="N7" s="59" t="s">
+        <v>175</v>
+      </c>
+      <c r="O7" s="63"/>
+      <c r="P7" s="67"/>
+    </row>
+    <row r="8" spans="1:16" ht="16.5">
+      <c r="A8" s="31">
         <v>3</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="35" t="s">
+      <c r="F8" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="G8" s="36" t="s">
+      <c r="G8" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="H8" s="37" t="s">
+      <c r="H8" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="I8" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="J8" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="38" t="s">
+      <c r="K8" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="39" t="s">
+      <c r="L8" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="M8" s="40" t="s">
+      <c r="M8" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N8" s="40"/>
-    </row>
-    <row r="9" spans="1:14" ht="13.5">
-      <c r="A9" s="33">
+      <c r="N8" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O8" s="64"/>
+      <c r="P8" s="68"/>
+    </row>
+    <row r="9" spans="1:16" ht="16.5">
+      <c r="A9" s="31">
         <v>4</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="34" t="s">
+      <c r="E9" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="35" t="s">
+      <c r="F9" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="G9" s="36" t="s">
+      <c r="G9" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="I9" s="34" t="s">
+      <c r="I9" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="J9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K9" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="39" t="s">
+      <c r="L9" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="M9" s="40" t="s">
+      <c r="M9" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N9" s="40"/>
-    </row>
-    <row r="10" spans="1:14" ht="13.5">
-      <c r="A10" s="42">
+      <c r="N9" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O9" s="64"/>
+      <c r="P9" s="68"/>
+    </row>
+    <row r="10" spans="1:16" ht="16.5">
+      <c r="A10" s="38">
         <v>5</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="43" t="s">
+      <c r="D10" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="43" t="s">
+      <c r="E10" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="45" t="s">
+      <c r="G10" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="45" t="s">
+      <c r="H10" s="41" t="s">
         <v>161</v>
       </c>
-      <c r="I10" s="43" t="s">
+      <c r="I10" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="43" t="s">
+      <c r="J10" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="K10" s="38" t="s">
+      <c r="K10" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="L10" s="39" t="s">
+      <c r="L10" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="M10" s="40" t="s">
+      <c r="M10" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N10" s="40"/>
-    </row>
-    <row r="11" spans="1:14" ht="13.5">
-      <c r="A11" s="33">
+      <c r="N10" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O10" s="64"/>
+      <c r="P10" s="68"/>
+    </row>
+    <row r="11" spans="1:16" ht="16.5">
+      <c r="A11" s="31">
         <v>8</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="G11" s="48" t="s">
+      <c r="G11" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="H11" s="37" t="s">
+      <c r="H11" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="I11" s="34" t="s">
+      <c r="I11" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="J11" s="34" t="s">
+      <c r="J11" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="38" t="s">
+      <c r="K11" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="39" t="s">
+      <c r="L11" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="M11" s="40" t="s">
+      <c r="M11" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N11" s="40"/>
-    </row>
-    <row r="12" spans="1:14" ht="13.5">
-      <c r="A12" s="33">
+      <c r="N11" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O11" s="64"/>
+      <c r="P11" s="68"/>
+    </row>
+    <row r="12" spans="1:16" ht="13.5">
+      <c r="A12" s="31">
         <v>20</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F12" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="37" t="s">
+      <c r="G12" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="H12" s="37" t="s">
+      <c r="H12" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="34" t="s">
+      <c r="I12" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="J12" s="34" t="s">
+      <c r="J12" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="K12" s="34" t="s">
+      <c r="K12" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="L12" s="39" t="s">
+      <c r="L12" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="M12" s="49" t="s">
+      <c r="M12" s="45" t="s">
         <v>167</v>
       </c>
-      <c r="N12" s="49"/>
-    </row>
-    <row r="13" spans="1:14" ht="40.5">
-      <c r="A13" s="33">
+      <c r="N12" s="45" t="s">
+        <v>171</v>
+      </c>
+      <c r="O12" s="64"/>
+      <c r="P12" s="68"/>
+    </row>
+    <row r="13" spans="1:16" ht="40.5">
+      <c r="A13" s="31">
         <v>6</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="34" t="s">
+      <c r="D13" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="34" t="s">
+      <c r="E13" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="35" t="s">
+      <c r="F13" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="37" t="s">
+      <c r="G13" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="H13" s="46" t="s">
+      <c r="H13" s="42" t="s">
         <v>159</v>
       </c>
-      <c r="I13" s="34" t="s">
+      <c r="I13" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="J13" s="34" t="s">
+      <c r="J13" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="K13" s="38" t="s">
+      <c r="K13" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="L13" s="39" t="s">
+      <c r="L13" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="M13" s="40" t="s">
+      <c r="M13" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N13" s="40"/>
-    </row>
-    <row r="14" spans="1:14" ht="40.5">
-      <c r="A14" s="42">
+      <c r="N13" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O13" s="64"/>
+      <c r="P13" s="68"/>
+    </row>
+    <row r="14" spans="1:16" ht="40.5">
+      <c r="A14" s="38">
         <v>7</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="43" t="s">
+      <c r="C14" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="F14" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="G14" s="45" t="s">
+      <c r="G14" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="H14" s="47" t="s">
+      <c r="H14" s="43" t="s">
         <v>158</v>
       </c>
-      <c r="I14" s="43" t="s">
+      <c r="I14" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="J14" s="43" t="s">
+      <c r="J14" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="K14" s="38" t="s">
+      <c r="K14" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="L14" s="39" t="s">
+      <c r="L14" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="M14" s="40" t="s">
+      <c r="M14" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N14" s="40"/>
-    </row>
-    <row r="15" spans="1:14" ht="13.5">
-      <c r="A15" s="33">
+      <c r="N14" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O14" s="64"/>
+      <c r="P14" s="68"/>
+    </row>
+    <row r="15" spans="1:16" ht="16.5">
+      <c r="A15" s="31">
         <v>16</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="34" t="s">
+      <c r="E15" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="35" t="s">
+      <c r="F15" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="G15" s="37" t="s">
+      <c r="G15" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="H15" s="37" t="s">
+      <c r="H15" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="I15" s="34" t="s">
+      <c r="I15" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="K15" s="38" t="s">
+      <c r="K15" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="L15" s="39" t="s">
+      <c r="L15" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="M15" s="40" t="s">
+      <c r="M15" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N15" s="40"/>
-    </row>
-    <row r="16" spans="1:14" ht="13.5">
-      <c r="A16" s="33">
+      <c r="N15" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="O15" s="64" t="s">
+        <v>179</v>
+      </c>
+      <c r="P15" s="68" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="13.5">
+      <c r="A16" s="31">
         <v>17</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="35" t="s">
+      <c r="F16" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="G16" s="37" t="s">
+      <c r="G16" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="H16" s="37" t="s">
+      <c r="H16" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="I16" s="34" t="s">
+      <c r="I16" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="K16" s="34" t="s">
+      <c r="K16" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="L16" s="39" t="s">
+      <c r="L16" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="M16" s="40" t="s">
+      <c r="M16" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="N16" s="40"/>
-    </row>
-    <row r="17" spans="1:14" ht="13.5">
-      <c r="A17" s="33">
+      <c r="N16" s="60" t="s">
+        <v>175</v>
+      </c>
+      <c r="O16" s="64"/>
+      <c r="P16" s="68"/>
+    </row>
+    <row r="17" spans="1:16" ht="16.5">
+      <c r="A17" s="31">
         <v>19</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" s="35" t="s">
+      <c r="E17" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="F17" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="G17" s="37" t="s">
+      <c r="G17" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="H17" s="37" t="s">
+      <c r="H17" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="I17" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="J17" s="34" t="s">
+      <c r="I17" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="J17" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="L17" s="39" t="s">
+      <c r="K17" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="L17" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="M17" s="49" t="s">
+      <c r="M17" s="45" t="s">
         <v>167</v>
       </c>
-      <c r="N17" s="49"/>
-    </row>
-    <row r="18" spans="1:14" ht="13.5">
-      <c r="A18" s="50">
+      <c r="N17" s="45" t="s">
+        <v>171</v>
+      </c>
+      <c r="O17" s="64"/>
+      <c r="P17" s="68"/>
+    </row>
+    <row r="18" spans="1:16" ht="16.5">
+      <c r="A18" s="46">
         <v>1</v>
       </c>
-      <c r="B18" s="51" t="s">
+      <c r="B18" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="51" t="s">
+      <c r="C18" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="51" t="s">
+      <c r="D18" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="51" t="s">
+      <c r="E18" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="F18" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="G18" s="53" t="s">
+      <c r="G18" s="49" t="s">
         <v>112</v>
       </c>
-      <c r="H18" s="52" t="s">
+      <c r="H18" s="48" t="s">
         <v>169</v>
       </c>
-      <c r="I18" s="51" t="s">
+      <c r="I18" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="51" t="s">
+      <c r="J18" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="K18" s="54" t="s">
+      <c r="K18" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="L18" s="55" t="s">
+      <c r="L18" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="M18" s="56" t="s">
+      <c r="M18" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="N18" s="56"/>
-    </row>
-    <row r="19" spans="1:14" ht="13.5">
-      <c r="A19" s="50">
+      <c r="N18" s="51" t="s">
+        <v>171</v>
+      </c>
+      <c r="O18" s="65"/>
+      <c r="P18" s="69"/>
+    </row>
+    <row r="19" spans="1:16" ht="16.5">
+      <c r="A19" s="46">
         <v>2</v>
       </c>
-      <c r="B19" s="51" t="s">
+      <c r="B19" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="51" t="s">
+      <c r="C19" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="51" t="s">
+      <c r="D19" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="51" t="s">
+      <c r="E19" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="52" t="s">
+      <c r="F19" s="48" t="s">
         <v>107</v>
       </c>
-      <c r="G19" s="53" t="s">
+      <c r="G19" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="H19" s="52"/>
-      <c r="I19" s="51" t="s">
+      <c r="H19" s="48"/>
+      <c r="I19" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="51" t="s">
+      <c r="J19" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="54" t="s">
+      <c r="K19" s="58" t="s">
         <v>47</v>
       </c>
-      <c r="L19" s="55" t="s">
+      <c r="L19" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="M19" s="56" t="s">
+      <c r="M19" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="N19" s="56"/>
-    </row>
-    <row r="20" spans="1:14" ht="13.5">
-      <c r="A20" s="50">
+      <c r="N19" s="51" t="s">
+        <v>171</v>
+      </c>
+      <c r="O19" s="65"/>
+      <c r="P19" s="69"/>
+    </row>
+    <row r="20" spans="1:16" ht="16.5">
+      <c r="A20" s="46">
         <v>15</v>
       </c>
-      <c r="B20" s="51" t="s">
+      <c r="B20" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="51" t="s">
+      <c r="C20" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="51" t="s">
+      <c r="D20" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="51" t="s">
+      <c r="E20" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="52" t="s">
+      <c r="F20" s="48" t="s">
         <v>130</v>
       </c>
-      <c r="G20" s="57" t="s">
+      <c r="G20" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="H20" s="57" t="s">
+      <c r="H20" s="52" t="s">
         <v>170</v>
       </c>
-      <c r="I20" s="51" t="s">
+      <c r="I20" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="J20" s="51" t="s">
+      <c r="J20" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="K20" s="54" t="s">
+      <c r="K20" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="L20" s="55" t="s">
+      <c r="L20" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="M20" s="56" t="s">
+      <c r="M20" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="N20" s="56"/>
-    </row>
-    <row r="21" spans="1:14" ht="13.5">
-      <c r="A21" s="50">
+      <c r="N20" s="51" t="s">
+        <v>171</v>
+      </c>
+      <c r="O20" s="65"/>
+      <c r="P20" s="69"/>
+    </row>
+    <row r="21" spans="1:16" ht="16.5">
+      <c r="A21" s="46">
         <v>18</v>
       </c>
-      <c r="B21" s="51" t="s">
+      <c r="B21" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="51" t="s">
+      <c r="C21" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="51" t="s">
+      <c r="D21" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="E21" s="51" t="s">
+      <c r="E21" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="52" t="s">
+      <c r="F21" s="48" t="s">
         <v>136</v>
       </c>
-      <c r="G21" s="57" t="s">
+      <c r="G21" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="H21" s="57" t="s">
+      <c r="H21" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="I21" s="51" t="s">
+      <c r="I21" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="J21" s="51" t="s">
+      <c r="J21" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="K21" s="54" t="s">
+      <c r="K21" s="58" t="s">
         <v>82</v>
       </c>
-      <c r="L21" s="55" t="s">
+      <c r="L21" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="M21" s="56" t="s">
+      <c r="M21" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="N21" s="56"/>
+      <c r="N21" s="51" t="s">
+        <v>171</v>
+      </c>
+      <c r="O21" s="65"/>
+      <c r="P21" s="69"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N21" xr:uid="{2C0977FD-8DA5-49F0-81F0-04370578922E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M23">
     <sortCondition ref="M2:M23"/>
     <sortCondition descending="1" ref="L2:L23"/>
@@ -3104,6 +3295,16 @@
     <hyperlink ref="F21" r:id="rId25" xr:uid="{679D3E72-9279-47D3-91CD-99C8523C3DEA}"/>
     <hyperlink ref="F17" r:id="rId26" xr:uid="{92BCAE65-3EDC-4C7F-8029-BAF238008192}"/>
     <hyperlink ref="F12" r:id="rId27" xr:uid="{22EC201B-FDE9-42C4-9650-3D081C48AAC0}"/>
+    <hyperlink ref="K3" r:id="rId28" xr:uid="{698CBA0F-06F3-4922-9779-E12B3D2FD331}"/>
+    <hyperlink ref="K4" r:id="rId29" xr:uid="{1F3CA864-0B3B-4263-A942-414BF6278292}"/>
+    <hyperlink ref="K5" r:id="rId30" xr:uid="{ABE87F78-8AB3-4A32-8559-E56F40B7FBD3}"/>
+    <hyperlink ref="K6" r:id="rId31" xr:uid="{EBBE1435-CCCC-4856-B7C7-22D2BEA31546}"/>
+    <hyperlink ref="K8" r:id="rId32" xr:uid="{D2F7D64A-0EAF-48A1-B9CE-133306CAFD60}"/>
+    <hyperlink ref="K9" r:id="rId33" xr:uid="{B126A3EF-010E-4FFD-AB39-9064F86BE6D6}"/>
+    <hyperlink ref="K10" r:id="rId34" xr:uid="{4C103A31-3009-44FA-9DFA-98D69942D9A9}"/>
+    <hyperlink ref="K17" r:id="rId35" xr:uid="{412663CF-D238-4C74-BF18-0B5FF19A2E8E}"/>
+    <hyperlink ref="K18" r:id="rId36" xr:uid="{DC8AE4E3-CF09-492A-B698-CD64497C7054}"/>
+    <hyperlink ref="K20" r:id="rId37" xr:uid="{522720C3-B84A-4C46-AC49-D3CFBC73CE3C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 17:26:24
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
+++ b/vault/50_FGI/FGI 업계/대구석 관련 협업사 리스트.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3045BADB-B8AE-4BD1-A4BE-A0CE561D7D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563E5252-3665-4486-8A61-B1B9D8600944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" tabRatio="221" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="221" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="국디마 업데이트" sheetId="17" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="183">
   <si>
     <t>일련
 번호</t>
@@ -748,11 +748,19 @@
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
-    <t>불참 확정</t>
-    <phoneticPr fontId="9" type="noConversion"/>
-  </si>
-  <si>
     <t>1차 전화컨택</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>불참회신</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>참석회신</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>불참회신</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -2326,7 +2334,7 @@
         <v>178</v>
       </c>
       <c r="P1" s="66" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="16.5">
@@ -2876,7 +2884,9 @@
       <c r="N13" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="O13" s="64"/>
+      <c r="O13" s="64" t="s">
+        <v>180</v>
+      </c>
       <c r="P13" s="68"/>
     </row>
     <row r="14" spans="1:16" ht="40.5">
@@ -2922,7 +2932,9 @@
       <c r="N14" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="O14" s="64"/>
+      <c r="O14" s="64" t="s">
+        <v>181</v>
+      </c>
       <c r="P14" s="68"/>
     </row>
     <row r="15" spans="1:16" ht="16.5">
@@ -2969,7 +2981,7 @@
         <v>171</v>
       </c>
       <c r="O15" s="64" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="P15" s="68" t="s">
         <v>84</v>
@@ -3110,7 +3122,9 @@
       <c r="N18" s="51" t="s">
         <v>171</v>
       </c>
-      <c r="O18" s="65"/>
+      <c r="O18" s="65" t="s">
+        <v>181</v>
+      </c>
       <c r="P18" s="69"/>
     </row>
     <row r="19" spans="1:16" ht="16.5">

</xml_diff>